<commit_message>
Confirm ITUK/MIDI SAP codes and Belgium sub-market roll-up
Per Jerome's confirmation: SAP code 2194 is ITUK (not MIDI as the old
build script assumed); MIDI has no SAP sold-to code with us at all;
Netherlands/Poland/Luxembourg are confirmed sub-markets under Belgium
(IBX) with no separate codes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XMV1DqJ3388g2AcSD6uzkT
</commit_message>
<xml_diff>
--- a/03_analytics/Isuzu/prism/data/db_name_and_sold_to_mapping.xlsx
+++ b/03_analytics/Isuzu/prism/data/db_name_and_sold_to_mapping.xlsx
@@ -972,7 +972,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>2575</t>
+          <t>2575 / 2194</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr"/>
@@ -1157,11 +1157,7 @@
           <t>CV+LCV</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>88</t>
-        </is>
-      </c>
+      <c r="F18" s="5" t="inlineStr"/>
       <c r="G18" s="5" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr">
         <is>
@@ -1170,7 +1166,7 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>No usable ISZE sales data — see question below</t>
+          <t>No SAP sold-to code — no usable ISZE sales data</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Turkey/AIOS code 77 and track two unidentified SAP codes
Jerome confirmed: SAP code 77 is AIOS (Anadolu Isuzu Otomotiv Sanayi,
the Turkey legal entity) — not an ISZE customer, kept for reference.
Codes 373 and 2970 remain unidentified; added as explicit UNKNOWN rows
rather than left undocumented.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XMV1DqJ3388g2AcSD6uzkT
</commit_message>
<xml_diff>
--- a/03_analytics/Isuzu/prism/data/db_name_and_sold_to_mapping.xlsx
+++ b/03_analytics/Isuzu/prism/data/db_name_and_sold_to_mapping.xlsx
@@ -10,7 +10,7 @@
     <sheet name="DB Name &amp; Code Mapping" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DB Name &amp; Code Mapping'!$A$1:$I$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DB Name &amp; Code Mapping'!$A$1:$I$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="42" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -1446,7 +1446,11 @@
           <t>ANADOLU ISUZU OTOMOTIV</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr"/>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>AIOS</t>
+        </is>
+      </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Turkey</t>
@@ -1457,7 +1461,11 @@
           <t>CV+LCV</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr"/>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
       <c r="G26" s="5" t="inlineStr"/>
       <c r="H26" s="4" t="inlineStr">
         <is>
@@ -1466,7 +1474,7 @@
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>Not an ISZE customer</t>
+          <t>Not an ISZE customer — kept for reference</t>
         </is>
       </c>
     </row>
@@ -1684,8 +1692,62 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr"/>
+      <c r="C33" s="5" t="inlineStr"/>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr"/>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>373</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Unidentified</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>Not identified — 2 lines seen in billing</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr"/>
+      <c r="C34" s="5" t="inlineStr"/>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="4" t="inlineStr"/>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>2970</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr"/>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Unidentified</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Not identified — 1 line seen in billing</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I32"/>
+  <autoFilter ref="A1:I34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resolve codes 373 and 2970 via full FY23-26 billing scan; flag MIDI discrepancy
Ran a full scan across the three CY billing exports available in this
session (2023-2024, old 2025, Q1 2026 — ~476k lines combined) instead
of the earlier small export sample:
- 373 = ISUZU MOTORS INT OPERATIONS (internal/HQ entity, not a country
  distributor)
- 2970 = Forlog NV (already-known excluded micro account) — merged
  into the existing FORLOG_EXCLUDE row
- Re-confirmed 2194 = ITUK and 77 = AIOS/Turkey at full-dataset scale
  (not just the earlier sample)
- Flagged a real discrepancy: the full scan shows 6,635 lines billed
  under "MIDI EUROPE S.R.L." at code 88 across FY23-26, which conflicts
  with Jerome's note that MIDI has no code with us. Left MIDI's code
  blank per his correction, noted the conflict for a second look.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XMV1DqJ3388g2AcSD6uzkT
</commit_message>
<xml_diff>
--- a/03_analytics/Isuzu/prism/data/db_name_and_sold_to_mapping.xlsx
+++ b/03_analytics/Isuzu/prism/data/db_name_and_sold_to_mapping.xlsx
@@ -10,7 +10,7 @@
     <sheet name="DB Name &amp; Code Mapping" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DB Name &amp; Code Mapping'!$A$1:$I$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DB Name &amp; Code Mapping'!$A$1:$I$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,10 +466,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -477,7 +477,7 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>No SAP sold-to code — no usable ISZE sales data</t>
+          <t>No SAP sold-to code per Jerome (2026-08-11) — flag: full FY23-26 billing scan shows 6,635 lines under this name at code 88, worth a second look if that volume matters</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr"/>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>2970</t>
+        </is>
+      </c>
       <c r="G32" s="5" t="inlineStr"/>
       <c r="H32" s="4" t="inlineStr">
         <is>
@@ -1695,13 +1699,21 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr"/>
+          <t>ISUZU_INT_OPERATIONS</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>ISUZU MOTORS INT OPERATIONS</t>
+        </is>
+      </c>
       <c r="C33" s="5" t="inlineStr"/>
       <c r="D33" s="5" t="inlineStr"/>
-      <c r="E33" s="4" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
           <t>373</t>
@@ -1710,44 +1722,17 @@
       <c r="G33" s="5" t="inlineStr"/>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Unidentified</t>
+          <t>Excluded</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>Not identified — 2 lines seen in billing</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr"/>
-      <c r="C34" s="5" t="inlineStr"/>
-      <c r="D34" s="5" t="inlineStr"/>
-      <c r="E34" s="4" t="inlineStr"/>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>2970</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr"/>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>Unidentified</t>
-        </is>
-      </c>
-      <c r="I34" s="5" t="inlineStr">
-        <is>
-          <t>Not identified — 1 line seen in billing</t>
+          <t>Internal/HQ operations entity, not a country distributor — 1 line seen in billing</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I34"/>
+  <autoFilter ref="A1:I33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>